<commit_message>
Poprawiona odpowiedź na pytanie d1-28
</commit_message>
<xml_diff>
--- a/UKE_porownanie_pytan.xlsx
+++ b/UKE_porownanie_pytan.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rafal\PycharmProjects\skrypty\UKE-nowe-pytania\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D87C400E-72C7-4370-BC2F-69049B03B980}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4FBCDE5-9F3E-4007-A08E-58DD4FE2A39C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TYTUL" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14580" uniqueCount="3497">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14583" uniqueCount="3500">
   <si>
     <r>
       <t xml:space="preserve">Siła elektromotoryczna ogniwa wynosi 1,5 V. </t>
@@ -28401,6 +28401,15 @@
   <si>
     <t>[mrkobel] Za Wikipedią:
 https://en.wikipedia.org/wiki/Maximum_usable_frequency</t>
+  </si>
+  <si>
+    <t>Poprawione po rozmowie [Maciejem Przezwickim]</t>
+  </si>
+  <si>
+    <t>Wersja:</t>
+  </si>
+  <si>
+    <t>Wersja z dnia 2026-01-13</t>
   </si>
 </sst>
 </file>
@@ -28870,7 +28879,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="48" bestFit="1" customWidth="1"/>
@@ -28888,184 +28897,192 @@
         <v>3454</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>3498</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>3499</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B3" s="1"/>
-    </row>
-    <row r="4" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+      <c r="B4" s="1"/>
+    </row>
+    <row r="5" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
         <v>3426</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B5" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+    <row r="6" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B6" s="1" t="s">
         <v>8</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>3425</v>
+        <v>16</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
+        <v>3425</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B9" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="60" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
+    <row r="10" spans="1:5" ht="60" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
         <v>3461</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B10" s="1" t="s">
         <v>3460</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
+    <row r="11" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
         <v>3493</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B11" s="1" t="s">
         <v>3492</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B12" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="C13" s="5" t="s">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C14" s="5" t="s">
         <v>3424</v>
       </c>
-      <c r="D13" s="5" t="s">
+      <c r="D14" s="5" t="s">
         <v>3446</v>
       </c>
-      <c r="E13" s="5" t="s">
+      <c r="E14" s="5" t="s">
         <v>3453</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="D14" s="9">
-        <f>COUNTIFS(porownanie!K:K,TYTUL!C14,porownanie!L:L,"A")</f>
-        <v>184</v>
-      </c>
-      <c r="E14" s="9">
-        <f>COUNTIFS(porownanie!K:K,TYTUL!C14,porownanie!M:M,"C")</f>
-        <v>139</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C15" s="7" t="s">
-        <v>21</v>
+        <v>13</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>22</v>
       </c>
       <c r="D15" s="9">
         <f>COUNTIFS(porownanie!K:K,TYTUL!C15,porownanie!L:L,"A")</f>
-        <v>224</v>
+        <v>184</v>
       </c>
       <c r="E15" s="9">
         <f>COUNTIFS(porownanie!K:K,TYTUL!C15,porownanie!M:M,"C")</f>
-        <v>142</v>
+        <v>139</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="C16" s="6" t="s">
-        <v>20</v>
+        <v>12</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>21</v>
       </c>
       <c r="D16" s="9">
         <f>COUNTIFS(porownanie!K:K,TYTUL!C16,porownanie!L:L,"A")</f>
-        <v>147</v>
+        <v>224</v>
       </c>
       <c r="E16" s="9">
         <f>COUNTIFS(porownanie!K:K,TYTUL!C16,porownanie!M:M,"C")</f>
-        <v>63</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B17" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="C17" s="8" t="s">
-        <v>23</v>
+        <v>11</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>20</v>
       </c>
       <c r="D17" s="9">
         <f>COUNTIFS(porownanie!K:K,TYTUL!C17,porownanie!L:L,"A")</f>
-        <v>108</v>
+        <v>147</v>
       </c>
       <c r="E17" s="9">
         <f>COUNTIFS(porownanie!K:K,TYTUL!C17,porownanie!M:M,"C")</f>
+        <v>63</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C18" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="D18" s="9">
+        <f>COUNTIFS(porownanie!K:K,TYTUL!C18,porownanie!L:L,"A")</f>
+        <v>108</v>
+      </c>
+      <c r="E18" s="9">
+        <f>COUNTIFS(porownanie!K:K,TYTUL!C18,porownanie!M:M,"C")</f>
         <v>89</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="C18" s="5" t="s">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C19" s="5" t="s">
         <v>3423</v>
       </c>
-      <c r="D18" s="5">
-        <f>SUM(D14:D17)</f>
+      <c r="D19" s="5">
+        <f>SUM(D15:D18)</f>
         <v>663</v>
       </c>
-      <c r="E18" s="5">
-        <f>SUM(E14:E17)</f>
+      <c r="E19" s="5">
+        <f>SUM(E15:E18)</f>
         <v>433</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B4" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="B5" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="B6" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
-    <hyperlink ref="B7" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
-    <hyperlink ref="B8" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
-    <hyperlink ref="B11" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="B5" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="B6" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="B7" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="B8" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="B9" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="B12" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -30193,9 +30210,11 @@
         <v>613</v>
       </c>
       <c r="I29" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="J29" s="2"/>
+        <v>37</v>
+      </c>
+      <c r="J29" s="2" t="s">
+        <v>3497</v>
+      </c>
       <c r="K29" s="7" t="s">
         <v>21</v>
       </c>
@@ -67837,7 +67856,7 @@
         <v>613</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="G30" s="1"/>
       <c r="H30" s="1" t="s">

</xml_diff>

<commit_message>
Poprawione odpowiedzi na pytania D1-160 i D1-170
Poprawione odpowiedzi na pytania D1-160 i D1-170
</commit_message>
<xml_diff>
--- a/UKE_porownanie_pytan.xlsx
+++ b/UKE_porownanie_pytan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rafal\PycharmProjects\skrypty\UKE-nowe-pytania\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{985788D3-F726-480C-AAB2-B34B7C71379E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E94BF693-DEA1-441C-8FF9-2837BFCA9E03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28409,10 +28409,10 @@
     <t>Wersja:</t>
   </si>
   <si>
-    <t>Poprawione przez Andrzeja K.</t>
-  </si>
-  <si>
     <t>Wersja z dnia 2026-03-22 v2</t>
+  </si>
+  <si>
+    <t>Poprawione przez andrekomor (https://github.com/andrekomor)</t>
   </si>
 </sst>
 </file>
@@ -28905,7 +28905,7 @@
         <v>3498</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>3500</v>
+        <v>3499</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -35783,7 +35783,7 @@
         <v>35</v>
       </c>
       <c r="J168" s="2" t="s">
-        <v>3499</v>
+        <v>3500</v>
       </c>
       <c r="K168" s="7" t="s">
         <v>21</v>
@@ -36161,7 +36161,7 @@
         <v>36</v>
       </c>
       <c r="J178" s="2" t="s">
-        <v>3499</v>
+        <v>3500</v>
       </c>
       <c r="K178" s="7" t="s">
         <v>21</v>

</xml_diff>

<commit_message>
Poprawione D1-160,170 ,289 i D2-39
Poprawione D1-160,170 ,289 i D2-39
</commit_message>
<xml_diff>
--- a/UKE_porownanie_pytan.xlsx
+++ b/UKE_porownanie_pytan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rafal\PycharmProjects\skrypty\UKE-nowe-pytania\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E94BF693-DEA1-441C-8FF9-2837BFCA9E03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1777D7C-E75E-40B4-897D-9CA5EC38202C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14593" uniqueCount="3501">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14596" uniqueCount="3500">
   <si>
     <r>
       <t xml:space="preserve">Siła elektromotoryczna ogniwa wynosi 1,5 V. </t>
@@ -27553,9 +27553,6 @@
     <t>Długość fali wynosi 1500 metrów. Jaka jest częstotliwość tej fali?</t>
   </si>
   <si>
-    <t>Zmiana kolejności odpowiedzi w stosunku do starego d2-234</t>
-  </si>
-  <si>
     <t>Zmiana treści w stosunku do starego d2-226</t>
   </si>
   <si>
@@ -28394,11 +28391,6 @@
     <t>[mrkobel] Prawidłowa odpowiedź to 2W (A, zamiast C). Również kalkulatory online podają taką odpowiedź jako prawidłową (np. https://www.everythingrf.com/rf-calculators/dbm-to-watts)</t>
   </si>
   <si>
-    <t>[mrkobel] wg. chat gpt prawidłowa odpowiedź to B.
-Więcej informacji również tutaj:
-https://sklep.delta.poznan.pl/dbi-zysk-energetyczny-anteny-izotropowej_l1_aid836.html</t>
-  </si>
-  <si>
     <t>[mrkobel] Za Wikipedią:
 https://en.wikipedia.org/wiki/Maximum_usable_frequency</t>
   </si>
@@ -28409,10 +28401,36 @@
     <t>Wersja:</t>
   </si>
   <si>
-    <t>Wersja z dnia 2026-03-22 v2</t>
-  </si>
-  <si>
     <t>Poprawione przez andrekomor (https://github.com/andrekomor)</t>
+  </si>
+  <si>
+    <t>Wersja z dnia 2026-03-22 v3</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <strike/>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>c</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>b</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -28897,15 +28915,15 @@
         <v>19</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>3454</v>
+        <v>3453</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
+        <v>3496</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>3498</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>3499</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -28916,7 +28934,7 @@
     </row>
     <row r="5" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>3426</v>
+        <v>3425</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>9</v>
@@ -28940,7 +28958,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>3425</v>
+        <v>3424</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>6</v>
@@ -28956,18 +28974,18 @@
     </row>
     <row r="10" spans="1:5" ht="60" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>3461</v>
+        <v>3460</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>3460</v>
+        <v>3459</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>3493</v>
+        <v>3492</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>3492</v>
+        <v>3491</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -28980,13 +28998,13 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C14" s="5" t="s">
-        <v>3424</v>
+        <v>3423</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>3446</v>
+        <v>3445</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>3453</v>
+        <v>3452</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
@@ -29067,7 +29085,7 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C19" s="5" t="s">
-        <v>3423</v>
+        <v>3422</v>
       </c>
       <c r="D19" s="5">
         <f>SUM(D15:D18)</f>
@@ -29116,10 +29134,10 @@
         <v>3089</v>
       </c>
       <c r="B1" s="5" t="s">
+        <v>3448</v>
+      </c>
+      <c r="C1" s="5" t="s">
         <v>3449</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>3450</v>
       </c>
       <c r="D1" s="5" t="s">
         <v>2358</v>
@@ -29146,16 +29164,16 @@
         <v>24</v>
       </c>
       <c r="L1" s="5" t="s">
+        <v>3450</v>
+      </c>
+      <c r="M1" s="12" t="s">
         <v>3451</v>
       </c>
-      <c r="M1" s="12" t="s">
-        <v>3452</v>
-      </c>
       <c r="N1" s="12" t="s">
-        <v>3448</v>
+        <v>3447</v>
       </c>
       <c r="O1" s="12" t="s">
-        <v>3447</v>
+        <v>3446</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
@@ -29409,7 +29427,7 @@
         <v>37</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>3457</v>
+        <v>3456</v>
       </c>
       <c r="K8" s="7" t="s">
         <v>21</v>
@@ -29524,7 +29542,7 @@
         <v>35</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>3458</v>
+        <v>3457</v>
       </c>
       <c r="K11" s="7" t="s">
         <v>21</v>
@@ -29717,7 +29735,7 @@
         <v>36</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>3459</v>
+        <v>3458</v>
       </c>
       <c r="K16" s="7" t="s">
         <v>21</v>
@@ -29793,7 +29811,7 @@
         <v>35</v>
       </c>
       <c r="J18" s="2" t="s">
-        <v>3455</v>
+        <v>3454</v>
       </c>
       <c r="K18" s="7" t="s">
         <v>21</v>
@@ -30099,7 +30117,7 @@
         <v>37</v>
       </c>
       <c r="J26" s="2" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="K26" s="7" t="s">
         <v>21</v>
@@ -30175,7 +30193,7 @@
         <v>36</v>
       </c>
       <c r="J28" s="2" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="K28" s="7" t="s">
         <v>21</v>
@@ -30216,7 +30234,7 @@
         <v>37</v>
       </c>
       <c r="J29" s="2" t="s">
-        <v>3497</v>
+        <v>3495</v>
       </c>
       <c r="K29" s="7" t="s">
         <v>21</v>
@@ -30407,7 +30425,7 @@
         <v>37</v>
       </c>
       <c r="J34" s="2" t="s">
-        <v>3463</v>
+        <v>3462</v>
       </c>
       <c r="K34" s="7" t="s">
         <v>21</v>
@@ -30487,7 +30505,7 @@
         <v>35</v>
       </c>
       <c r="J36" s="2" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="K36" s="7" t="s">
         <v>21</v>
@@ -30563,7 +30581,7 @@
         <v>37</v>
       </c>
       <c r="J38" s="2" t="s">
-        <v>3464</v>
+        <v>3463</v>
       </c>
       <c r="K38" s="7" t="s">
         <v>21</v>
@@ -30678,7 +30696,7 @@
         <v>36</v>
       </c>
       <c r="J41" s="2" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="K41" s="7" t="s">
         <v>21</v>
@@ -30834,7 +30852,7 @@
         <v>36</v>
       </c>
       <c r="J45" s="2" t="s">
-        <v>3466</v>
+        <v>3465</v>
       </c>
       <c r="K45" s="7" t="s">
         <v>21</v>
@@ -30914,7 +30932,7 @@
         <v>37</v>
       </c>
       <c r="J47" s="2" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="K47" s="7" t="s">
         <v>21</v>
@@ -30951,7 +30969,7 @@
         <v>36</v>
       </c>
       <c r="J48" s="2" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="K48" s="7" t="s">
         <v>21</v>
@@ -31027,7 +31045,7 @@
         <v>36</v>
       </c>
       <c r="J50" s="2" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="K50" s="7" t="s">
         <v>21</v>
@@ -31064,7 +31082,7 @@
         <v>35</v>
       </c>
       <c r="J51" s="2" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="K51" s="7" t="s">
         <v>21</v>
@@ -31220,7 +31238,7 @@
         <v>36</v>
       </c>
       <c r="J55" s="2" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="K55" s="7" t="s">
         <v>21</v>
@@ -31257,7 +31275,7 @@
         <v>37</v>
       </c>
       <c r="J56" s="2" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="K56" s="7" t="s">
         <v>21</v>
@@ -31448,7 +31466,7 @@
         <v>37</v>
       </c>
       <c r="J61" s="2" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="K61" s="7" t="s">
         <v>21</v>
@@ -31489,7 +31507,7 @@
         <v>37</v>
       </c>
       <c r="J62" s="2" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="K62" s="7" t="s">
         <v>21</v>
@@ -31600,7 +31618,7 @@
         <v>36</v>
       </c>
       <c r="J65" s="2" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="K65" s="7" t="s">
         <v>21</v>
@@ -33336,7 +33354,7 @@
         <v>36</v>
       </c>
       <c r="J107" s="2" t="s">
-        <v>3467</v>
+        <v>3466</v>
       </c>
       <c r="K107" s="7" t="s">
         <v>21</v>
@@ -33924,7 +33942,7 @@
         <v>37</v>
       </c>
       <c r="J121" s="2" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="K121" s="7" t="s">
         <v>21</v>
@@ -35103,7 +35121,7 @@
         <v>39</v>
       </c>
       <c r="J150" s="2" t="s">
-        <v>3494</v>
+        <v>3493</v>
       </c>
       <c r="K150" s="8" t="s">
         <v>23</v>
@@ -35783,7 +35801,7 @@
         <v>35</v>
       </c>
       <c r="J168" s="2" t="s">
-        <v>3500</v>
+        <v>3497</v>
       </c>
       <c r="K168" s="7" t="s">
         <v>21</v>
@@ -35935,7 +35953,7 @@
         <v>36</v>
       </c>
       <c r="J172" s="2" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="K172" s="7" t="s">
         <v>21</v>
@@ -36161,7 +36179,7 @@
         <v>36</v>
       </c>
       <c r="J178" s="2" t="s">
-        <v>3500</v>
+        <v>3497</v>
       </c>
       <c r="K178" s="7" t="s">
         <v>21</v>
@@ -36198,7 +36216,7 @@
         <v>36</v>
       </c>
       <c r="J179" s="2" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="K179" s="7" t="s">
         <v>21</v>
@@ -37871,7 +37889,7 @@
         <v>36</v>
       </c>
       <c r="J224" s="2" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="K224" s="7" t="s">
         <v>21</v>
@@ -37953,7 +37971,7 @@
         <v>35</v>
       </c>
       <c r="J226" s="2" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="K226" s="7" t="s">
         <v>21</v>
@@ -38382,7 +38400,7 @@
         <v>37</v>
       </c>
       <c r="J237" s="2" t="s">
-        <v>3465</v>
+        <v>3464</v>
       </c>
       <c r="K237" s="7" t="s">
         <v>21</v>
@@ -38456,7 +38474,7 @@
         <v>35</v>
       </c>
       <c r="J239" s="2" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="K239" s="7" t="s">
         <v>21</v>
@@ -38729,7 +38747,7 @@
         <v>35</v>
       </c>
       <c r="J246" s="2" t="s">
-        <v>3468</v>
+        <v>3467</v>
       </c>
       <c r="K246" s="7" t="s">
         <v>21</v>
@@ -38805,7 +38823,7 @@
         <v>35</v>
       </c>
       <c r="J248" s="2" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="K248" s="7" t="s">
         <v>21</v>
@@ -38881,7 +38899,7 @@
         <v>35</v>
       </c>
       <c r="J250" s="2" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="K250" s="7" t="s">
         <v>21</v>
@@ -39066,7 +39084,7 @@
         <v>35</v>
       </c>
       <c r="J255" s="2" t="s">
-        <v>3487</v>
+        <v>3486</v>
       </c>
       <c r="K255" s="7" t="s">
         <v>21</v>
@@ -39181,7 +39199,7 @@
         <v>35</v>
       </c>
       <c r="J258" s="2" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="K258" s="7" t="s">
         <v>21</v>
@@ -39218,7 +39236,7 @@
         <v>36</v>
       </c>
       <c r="J259" s="2" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="K259" s="7" t="s">
         <v>21</v>
@@ -39290,7 +39308,7 @@
         <v>35</v>
       </c>
       <c r="J261" s="2" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="K261" s="7" t="s">
         <v>21</v>
@@ -39331,7 +39349,7 @@
         <v>35</v>
       </c>
       <c r="J262" s="2" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="K262" s="7" t="s">
         <v>21</v>
@@ -39407,7 +39425,7 @@
         <v>37</v>
       </c>
       <c r="J264" s="2" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="K264" s="7" t="s">
         <v>21</v>
@@ -39444,7 +39462,7 @@
         <v>36</v>
       </c>
       <c r="J265" s="2" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="K265" s="7" t="s">
         <v>21</v>
@@ -39481,7 +39499,7 @@
         <v>37</v>
       </c>
       <c r="J266" s="2" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="K266" s="7" t="s">
         <v>21</v>
@@ -39553,7 +39571,7 @@
         <v>37</v>
       </c>
       <c r="J268" s="2" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="K268" s="7" t="s">
         <v>21</v>
@@ -39590,7 +39608,7 @@
         <v>35</v>
       </c>
       <c r="J269" s="2" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="K269" s="7" t="s">
         <v>21</v>
@@ -39631,7 +39649,7 @@
         <v>37</v>
       </c>
       <c r="J270" s="2" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="K270" s="7" t="s">
         <v>21</v>
@@ -39668,7 +39686,7 @@
         <v>35</v>
       </c>
       <c r="J271" s="2" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="K271" s="7" t="s">
         <v>21</v>
@@ -39705,7 +39723,7 @@
         <v>36</v>
       </c>
       <c r="J272" s="2" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="K272" s="7" t="s">
         <v>21</v>
@@ -39816,7 +39834,7 @@
         <v>36</v>
       </c>
       <c r="J275" s="2" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="K275" s="7" t="s">
         <v>21</v>
@@ -39853,7 +39871,7 @@
         <v>36</v>
       </c>
       <c r="J276" s="2" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="K276" s="7" t="s">
         <v>21</v>
@@ -39962,7 +39980,7 @@
         <v>37</v>
       </c>
       <c r="J279" s="2" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="K279" s="7" t="s">
         <v>21</v>
@@ -39999,7 +40017,7 @@
         <v>36</v>
       </c>
       <c r="J280" s="2" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="K280" s="7" t="s">
         <v>21</v>
@@ -40036,7 +40054,7 @@
         <v>35</v>
       </c>
       <c r="J281" s="2" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="K281" s="7" t="s">
         <v>21</v>
@@ -40073,7 +40091,7 @@
         <v>37</v>
       </c>
       <c r="J282" s="2" t="s">
-        <v>3465</v>
+        <v>3464</v>
       </c>
       <c r="K282" s="7" t="s">
         <v>21</v>
@@ -40114,7 +40132,7 @@
         <v>35</v>
       </c>
       <c r="J283" s="2" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="K283" s="7" t="s">
         <v>21</v>
@@ -40151,7 +40169,7 @@
         <v>35</v>
       </c>
       <c r="J284" s="2" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="K284" s="7" t="s">
         <v>21</v>
@@ -40188,7 +40206,7 @@
         <v>37</v>
       </c>
       <c r="J285" s="2" t="s">
-        <v>3469</v>
+        <v>3468</v>
       </c>
       <c r="K285" s="7" t="s">
         <v>21</v>
@@ -40225,7 +40243,7 @@
         <v>36</v>
       </c>
       <c r="J286" s="2" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="K286" s="7" t="s">
         <v>21</v>
@@ -40297,7 +40315,7 @@
         <v>36</v>
       </c>
       <c r="J288" s="2" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="K288" s="7" t="s">
         <v>21</v>
@@ -40334,7 +40352,7 @@
         <v>36</v>
       </c>
       <c r="J289" s="2" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="K289" s="7" t="s">
         <v>21</v>
@@ -40375,7 +40393,7 @@
         <v>36</v>
       </c>
       <c r="J290" s="2" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="K290" s="7" t="s">
         <v>21</v>
@@ -40486,7 +40504,7 @@
         <v>37</v>
       </c>
       <c r="J293" s="2" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="K293" s="7" t="s">
         <v>21</v>
@@ -40523,7 +40541,7 @@
         <v>37</v>
       </c>
       <c r="J294" s="2" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="K294" s="7" t="s">
         <v>21</v>
@@ -40560,7 +40578,7 @@
         <v>36</v>
       </c>
       <c r="J295" s="2" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="K295" s="7" t="s">
         <v>21</v>
@@ -40601,7 +40619,7 @@
         <v>37</v>
       </c>
       <c r="J296" s="2" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="K296" s="7" t="s">
         <v>21</v>
@@ -40761,7 +40779,7 @@
         <v>35</v>
       </c>
       <c r="J300" s="2" t="s">
-        <v>3470</v>
+        <v>3469</v>
       </c>
       <c r="K300" s="7" t="s">
         <v>21</v>
@@ -40798,7 +40816,7 @@
         <v>36</v>
       </c>
       <c r="J301" s="2" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="K301" s="7" t="s">
         <v>21</v>
@@ -40835,7 +40853,7 @@
         <v>37</v>
       </c>
       <c r="J302" s="2" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="K302" s="7" t="s">
         <v>21</v>
@@ -40876,7 +40894,7 @@
         <v>36</v>
       </c>
       <c r="J303" s="2" t="s">
-        <v>3471</v>
+        <v>3470</v>
       </c>
       <c r="K303" s="7" t="s">
         <v>21</v>
@@ -40913,7 +40931,7 @@
         <v>36</v>
       </c>
       <c r="J304" s="2" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="K304" s="7" t="s">
         <v>21</v>
@@ -40929,7 +40947,7 @@
       </c>
       <c r="O304" s="9"/>
     </row>
-    <row r="305" spans="1:15" ht="75" x14ac:dyDescent="0.25">
+    <row r="305" spans="1:15" ht="45" x14ac:dyDescent="0.25">
       <c r="A305" s="1">
         <v>304</v>
       </c>
@@ -40951,10 +40969,10 @@
         <v>384</v>
       </c>
       <c r="I305" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="J305" s="2" t="s">
-        <v>3495</v>
+        <v>3497</v>
       </c>
       <c r="K305" s="7" t="s">
         <v>21</v>
@@ -40995,7 +41013,7 @@
         <v>36</v>
       </c>
       <c r="J306" s="2" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="K306" s="7" t="s">
         <v>21</v>
@@ -41034,7 +41052,7 @@
         <v>37</v>
       </c>
       <c r="J307" s="2" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="K307" s="8" t="s">
         <v>23</v>
@@ -41112,7 +41130,7 @@
         <v>37</v>
       </c>
       <c r="J309" s="2" t="s">
-        <v>3472</v>
+        <v>3471</v>
       </c>
       <c r="K309" s="7" t="s">
         <v>21</v>
@@ -41192,7 +41210,7 @@
         <v>35</v>
       </c>
       <c r="J311" s="2" t="s">
-        <v>3473</v>
+        <v>3472</v>
       </c>
       <c r="K311" s="7" t="s">
         <v>21</v>
@@ -41233,7 +41251,7 @@
         <v>37</v>
       </c>
       <c r="J312" s="2" t="s">
-        <v>3474</v>
+        <v>3473</v>
       </c>
       <c r="K312" s="7" t="s">
         <v>21</v>
@@ -41309,7 +41327,7 @@
         <v>37</v>
       </c>
       <c r="J314" s="2" t="s">
-        <v>3475</v>
+        <v>3474</v>
       </c>
       <c r="K314" s="7" t="s">
         <v>21</v>
@@ -41463,7 +41481,7 @@
         <v>37</v>
       </c>
       <c r="J318" s="2" t="s">
-        <v>3476</v>
+        <v>3475</v>
       </c>
       <c r="K318" s="7" t="s">
         <v>21</v>
@@ -41500,7 +41518,7 @@
         <v>35</v>
       </c>
       <c r="J319" s="2" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="K319" s="7" t="s">
         <v>21</v>
@@ -41619,7 +41637,7 @@
         <v>36</v>
       </c>
       <c r="J322" s="2" t="s">
-        <v>3496</v>
+        <v>3494</v>
       </c>
       <c r="K322" s="7" t="s">
         <v>21</v>
@@ -41660,7 +41678,7 @@
         <v>37</v>
       </c>
       <c r="J323" s="2" t="s">
-        <v>3485</v>
+        <v>3484</v>
       </c>
       <c r="K323" s="7" t="s">
         <v>21</v>
@@ -41857,7 +41875,7 @@
         <v>37</v>
       </c>
       <c r="J328" s="2" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="K328" s="7" t="s">
         <v>21</v>
@@ -41933,7 +41951,7 @@
         <v>36</v>
       </c>
       <c r="J330" s="2" t="s">
-        <v>3477</v>
+        <v>3476</v>
       </c>
       <c r="K330" s="7" t="s">
         <v>21</v>
@@ -42091,7 +42109,7 @@
         <v>37</v>
       </c>
       <c r="J334" s="2" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="K334" s="7" t="s">
         <v>21</v>
@@ -42167,7 +42185,7 @@
         <v>36</v>
       </c>
       <c r="J336" s="2" t="s">
-        <v>3478</v>
+        <v>3477</v>
       </c>
       <c r="K336" s="7" t="s">
         <v>21</v>
@@ -42477,7 +42495,7 @@
         <v>37</v>
       </c>
       <c r="J344" s="2" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="K344" s="7" t="s">
         <v>21</v>
@@ -42592,7 +42610,7 @@
         <v>37</v>
       </c>
       <c r="J347" s="2" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="K347" s="7" t="s">
         <v>21</v>
@@ -42668,7 +42686,7 @@
         <v>37</v>
       </c>
       <c r="J349" s="2" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="K349" s="7" t="s">
         <v>21</v>
@@ -45436,7 +45454,7 @@
         <v>37</v>
       </c>
       <c r="J423" s="2" t="s">
-        <v>3479</v>
+        <v>3478</v>
       </c>
       <c r="K423" s="7" t="s">
         <v>21</v>
@@ -46500,10 +46518,12 @@
       <c r="H449" s="4" t="s">
         <v>250</v>
       </c>
-      <c r="I449" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="J449" s="4"/>
+      <c r="I449" s="14" t="s">
+        <v>3499</v>
+      </c>
+      <c r="J449" s="2" t="s">
+        <v>3497</v>
+      </c>
       <c r="K449" s="8" t="s">
         <v>23</v>
       </c>
@@ -50577,7 +50597,7 @@
         <v>36</v>
       </c>
       <c r="J552" s="2" t="s">
-        <v>3489</v>
+        <v>3488</v>
       </c>
       <c r="K552" s="7" t="s">
         <v>21</v>
@@ -50854,7 +50874,7 @@
         <v>37</v>
       </c>
       <c r="J559" s="2" t="s">
-        <v>3478</v>
+        <v>3477</v>
       </c>
       <c r="K559" s="7" t="s">
         <v>21</v>
@@ -51663,7 +51683,7 @@
         <v>35</v>
       </c>
       <c r="J580" s="2" t="s">
-        <v>3480</v>
+        <v>3479</v>
       </c>
       <c r="K580" s="7" t="s">
         <v>21</v>
@@ -52988,7 +53008,7 @@
         <v>36</v>
       </c>
       <c r="J611" s="2" t="s">
-        <v>3488</v>
+        <v>3487</v>
       </c>
       <c r="K611" s="7" t="s">
         <v>21</v>
@@ -53029,7 +53049,7 @@
         <v>35</v>
       </c>
       <c r="J612" s="2" t="s">
-        <v>3481</v>
+        <v>3480</v>
       </c>
       <c r="K612" s="7" t="s">
         <v>21</v>
@@ -53070,7 +53090,7 @@
         <v>36</v>
       </c>
       <c r="J613" s="2" t="s">
-        <v>3482</v>
+        <v>3481</v>
       </c>
       <c r="K613" s="7" t="s">
         <v>21</v>
@@ -53111,7 +53131,7 @@
         <v>36</v>
       </c>
       <c r="J614" s="2" t="s">
-        <v>3486</v>
+        <v>3485</v>
       </c>
       <c r="K614" s="7" t="s">
         <v>21</v>
@@ -53191,7 +53211,7 @@
         <v>35</v>
       </c>
       <c r="J616" s="2" t="s">
-        <v>3483</v>
+        <v>3482</v>
       </c>
       <c r="K616" s="7" t="s">
         <v>21</v>
@@ -54266,7 +54286,7 @@
         <v>35</v>
       </c>
       <c r="J643" s="2" t="s">
-        <v>3456</v>
+        <v>3455</v>
       </c>
       <c r="K643" s="7" t="s">
         <v>21</v>
@@ -54307,7 +54327,7 @@
         <v>36</v>
       </c>
       <c r="J644" s="2" t="s">
-        <v>3491</v>
+        <v>3490</v>
       </c>
       <c r="K644" s="7" t="s">
         <v>21</v>
@@ -54465,7 +54485,7 @@
         <v>36</v>
       </c>
       <c r="J648" s="2" t="s">
-        <v>3484</v>
+        <v>3483</v>
       </c>
       <c r="K648" s="7" t="s">
         <v>21</v>
@@ -54506,7 +54526,7 @@
         <v>36</v>
       </c>
       <c r="J649" s="2" t="s">
-        <v>3490</v>
+        <v>3489</v>
       </c>
       <c r="K649" s="7" t="s">
         <v>21</v>
@@ -54518,7 +54538,7 @@
         <v>594</v>
       </c>
       <c r="N649" s="9" t="s">
-        <v>3428</v>
+        <v>3427</v>
       </c>
       <c r="O649" s="9"/>
     </row>
@@ -55149,17 +55169,17 @@
       <c r="B666" s="1"/>
       <c r="C666" s="1"/>
       <c r="D666" s="2" t="s">
-        <v>3429</v>
+        <v>3428</v>
       </c>
       <c r="E666" s="1"/>
       <c r="F666" s="2" t="s">
+        <v>3429</v>
+      </c>
+      <c r="G666" s="2" t="s">
         <v>3430</v>
       </c>
-      <c r="G666" s="2" t="s">
+      <c r="H666" s="2" t="s">
         <v>3431</v>
-      </c>
-      <c r="H666" s="2" t="s">
-        <v>3432</v>
       </c>
       <c r="I666" s="2" t="s">
         <v>35</v>
@@ -55184,17 +55204,17 @@
       <c r="B667" s="1"/>
       <c r="C667" s="1"/>
       <c r="D667" s="2" t="s">
-        <v>3433</v>
+        <v>3432</v>
       </c>
       <c r="E667" s="1"/>
       <c r="F667" s="2" t="s">
+        <v>3433</v>
+      </c>
+      <c r="G667" s="2" t="s">
         <v>3434</v>
       </c>
-      <c r="G667" s="2" t="s">
+      <c r="H667" s="2" t="s">
         <v>3435</v>
-      </c>
-      <c r="H667" s="2" t="s">
-        <v>3436</v>
       </c>
       <c r="I667" s="2" t="s">
         <v>35</v>
@@ -55219,7 +55239,7 @@
       <c r="B668" s="1"/>
       <c r="C668" s="1"/>
       <c r="D668" s="2" t="s">
-        <v>3437</v>
+        <v>3436</v>
       </c>
       <c r="E668" s="1"/>
       <c r="F668" s="2">
@@ -55254,17 +55274,17 @@
       <c r="B669" s="1"/>
       <c r="C669" s="1"/>
       <c r="D669" s="2" t="s">
-        <v>3438</v>
+        <v>3437</v>
       </c>
       <c r="E669" s="1"/>
       <c r="F669" s="2" t="s">
+        <v>3438</v>
+      </c>
+      <c r="G669" s="2" t="s">
         <v>3439</v>
       </c>
-      <c r="G669" s="2" t="s">
+      <c r="H669" s="2" t="s">
         <v>3440</v>
-      </c>
-      <c r="H669" s="2" t="s">
-        <v>3441</v>
       </c>
       <c r="I669" s="2" t="s">
         <v>37</v>
@@ -55330,13 +55350,13 @@
         <v>41</v>
       </c>
       <c r="H1" s="5" t="s">
+        <v>3450</v>
+      </c>
+      <c r="I1" s="12" t="s">
         <v>3451</v>
       </c>
-      <c r="I1" s="12" t="s">
-        <v>3452</v>
-      </c>
       <c r="J1" s="12" t="s">
-        <v>3427</v>
+        <v>3426</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
@@ -67047,10 +67067,10 @@
   <sheetData>
     <row r="1" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
+        <v>3394</v>
+      </c>
+      <c r="B1" s="5" t="s">
         <v>3395</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>3396</v>
       </c>
       <c r="C1" s="5" t="s">
         <v>1699</v>
@@ -67068,21 +67088,21 @@
         <v>34</v>
       </c>
       <c r="H1" s="5" t="s">
+        <v>3450</v>
+      </c>
+      <c r="I1" s="12" t="s">
         <v>3451</v>
       </c>
-      <c r="I1" s="12" t="s">
-        <v>3452</v>
-      </c>
       <c r="J1" s="12" t="s">
-        <v>3427</v>
+        <v>3426</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>3445</v>
+        <v>3444</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>3422</v>
+        <v>3421</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -67287,7 +67307,7 @@
         <v>37</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>3457</v>
+        <v>3456</v>
       </c>
       <c r="H9" s="1" t="s">
         <v>1659</v>
@@ -67375,7 +67395,7 @@
         <v>35</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>3458</v>
+        <v>3457</v>
       </c>
       <c r="H12" s="1" t="s">
         <v>1659</v>
@@ -67418,7 +67438,7 @@
         <v>2779</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>3394</v>
+        <v>3393</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>1640</v>
@@ -67519,7 +67539,7 @@
         <v>36</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>3459</v>
+        <v>3458</v>
       </c>
       <c r="H17" s="1" t="s">
         <v>1659</v>
@@ -67577,7 +67597,7 @@
         <v>35</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>3455</v>
+        <v>3454</v>
       </c>
       <c r="H19" s="1" t="s">
         <v>1659</v>
@@ -67811,7 +67831,7 @@
         <v>37</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="H27" s="1" t="s">
         <v>1659</v>
@@ -67869,7 +67889,7 @@
         <v>36</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="H29" s="1" t="s">
         <v>1659</v>
@@ -67942,7 +67962,7 @@
         <v>2760</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>3393</v>
+        <v>3392</v>
       </c>
       <c r="C32" s="1" t="s">
         <v>1598</v>
@@ -68043,7 +68063,7 @@
         <v>37</v>
       </c>
       <c r="G35" s="1" t="s">
-        <v>3463</v>
+        <v>3462</v>
       </c>
       <c r="H35" s="1" t="s">
         <v>1659</v>
@@ -68105,7 +68125,7 @@
         <v>35</v>
       </c>
       <c r="G37" s="1" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="H37" s="1" t="s">
         <v>1659</v>
@@ -68163,7 +68183,7 @@
         <v>37</v>
       </c>
       <c r="G39" s="1" t="s">
-        <v>3464</v>
+        <v>3463</v>
       </c>
       <c r="H39" s="1" t="s">
         <v>1659</v>
@@ -68221,7 +68241,7 @@
         <v>36</v>
       </c>
       <c r="G41" s="1" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="H41" s="1" t="s">
         <v>1659</v>
@@ -68268,7 +68288,7 @@
         <v>2753</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>3392</v>
+        <v>3391</v>
       </c>
       <c r="C43" s="1" t="s">
         <v>1535</v>
@@ -68335,7 +68355,7 @@
         <v>36</v>
       </c>
       <c r="G45" s="1" t="s">
-        <v>3466</v>
+        <v>3465</v>
       </c>
       <c r="H45" s="1" t="s">
         <v>1659</v>
@@ -68397,7 +68417,7 @@
         <v>37</v>
       </c>
       <c r="G47" s="1" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="H47" s="1" t="s">
         <v>1659</v>
@@ -68425,7 +68445,7 @@
         <v>36</v>
       </c>
       <c r="G48" s="1" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="H48" s="1" t="s">
         <v>1659</v>
@@ -68483,7 +68503,7 @@
         <v>36</v>
       </c>
       <c r="G50" s="1" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="H50" s="1" t="s">
         <v>1659</v>
@@ -68511,7 +68531,7 @@
         <v>35</v>
       </c>
       <c r="G51" s="1" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="H51" s="1" t="s">
         <v>1659</v>
@@ -68631,7 +68651,7 @@
         <v>36</v>
       </c>
       <c r="G55" s="1" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="H55" s="1" t="s">
         <v>1659</v>
@@ -68659,7 +68679,7 @@
         <v>37</v>
       </c>
       <c r="G56" s="1" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="H56" s="1" t="s">
         <v>1659</v>
@@ -68805,7 +68825,7 @@
         <v>37</v>
       </c>
       <c r="G61" s="1" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="H61" s="1" t="s">
         <v>1659</v>
@@ -68837,7 +68857,7 @@
         <v>37</v>
       </c>
       <c r="G62" s="1" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="H62" s="1" t="s">
         <v>1659</v>
@@ -68921,7 +68941,7 @@
         <v>36</v>
       </c>
       <c r="G65" s="1" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="H65" s="1" t="s">
         <v>1659</v>
@@ -69119,7 +69139,7 @@
         <v>1118</v>
       </c>
       <c r="E72" s="1" t="s">
-        <v>3270</v>
+        <v>3269</v>
       </c>
       <c r="F72" s="1" t="s">
         <v>36</v>
@@ -69170,16 +69190,16 @@
         <v>2631</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>3391</v>
+        <v>3390</v>
       </c>
       <c r="C74" s="1" t="s">
-        <v>3332</v>
+        <v>3331</v>
       </c>
       <c r="D74" s="1" t="s">
-        <v>3301</v>
+        <v>3300</v>
       </c>
       <c r="E74" s="1" t="s">
-        <v>3269</v>
+        <v>3268</v>
       </c>
       <c r="F74" s="1" t="s">
         <v>36</v>
@@ -69209,7 +69229,7 @@
         <v>1115</v>
       </c>
       <c r="E75" s="1" t="s">
-        <v>3268</v>
+        <v>3267</v>
       </c>
       <c r="F75" s="1" t="s">
         <v>36</v>
@@ -69230,7 +69250,7 @@
         <v>2629</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>3390</v>
+        <v>3389</v>
       </c>
       <c r="C76" s="1" t="s">
         <v>1635</v>
@@ -69263,7 +69283,7 @@
         <v>2282</v>
       </c>
       <c r="C77" s="1" t="s">
-        <v>3320</v>
+        <v>3319</v>
       </c>
       <c r="D77" s="1" t="s">
         <v>1114</v>
@@ -69299,7 +69319,7 @@
         <v>1113</v>
       </c>
       <c r="E78" s="1" t="s">
-        <v>3267</v>
+        <v>3266</v>
       </c>
       <c r="F78" s="1" t="s">
         <v>36</v>
@@ -69350,7 +69370,7 @@
         <v>2729</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>3389</v>
+        <v>3388</v>
       </c>
       <c r="C80" s="1" t="s">
         <v>1631</v>
@@ -69380,13 +69400,13 @@
         <v>2728</v>
       </c>
       <c r="B81" s="1" t="s">
-        <v>3388</v>
+        <v>3387</v>
       </c>
       <c r="C81" s="1" t="s">
         <v>1413</v>
       </c>
       <c r="D81" s="1" t="s">
-        <v>3300</v>
+        <v>3299</v>
       </c>
       <c r="E81" s="1" t="s">
         <v>562</v>
@@ -69410,7 +69430,7 @@
         <v>2727</v>
       </c>
       <c r="B82" s="1" t="s">
-        <v>3421</v>
+        <v>3420</v>
       </c>
       <c r="C82" s="1" t="s">
         <v>1535</v>
@@ -69438,7 +69458,7 @@
         <v>2610</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>3387</v>
+        <v>3386</v>
       </c>
       <c r="C83" s="1" t="s">
         <v>1630</v>
@@ -69464,7 +69484,7 @@
         <v>2726</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>3386</v>
+        <v>3385</v>
       </c>
       <c r="C84" s="1" t="s">
         <v>3145</v>
@@ -69479,7 +69499,7 @@
         <v>36</v>
       </c>
       <c r="G84" s="1" t="s">
-        <v>3234</v>
+        <v>3233</v>
       </c>
       <c r="H84" s="1" t="s">
         <v>1659</v>
@@ -69522,10 +69542,10 @@
         <v>2725</v>
       </c>
       <c r="B86" s="1" t="s">
-        <v>3385</v>
+        <v>3384</v>
       </c>
       <c r="C86" s="1" t="s">
-        <v>3331</v>
+        <v>3330</v>
       </c>
       <c r="D86" s="1" t="s">
         <v>1105</v>
@@ -69555,7 +69575,7 @@
         <v>2271</v>
       </c>
       <c r="C87" s="1" t="s">
-        <v>3330</v>
+        <v>3329</v>
       </c>
       <c r="D87" s="1" t="s">
         <v>1104</v>
@@ -69672,7 +69692,7 @@
         <v>2605</v>
       </c>
       <c r="B91" s="1" t="s">
-        <v>3384</v>
+        <v>3383</v>
       </c>
       <c r="C91" s="1" t="s">
         <v>1622</v>
@@ -69814,7 +69834,7 @@
         <v>2602</v>
       </c>
       <c r="B96" s="1" t="s">
-        <v>3383</v>
+        <v>3382</v>
       </c>
       <c r="C96" s="1" t="s">
         <v>506</v>
@@ -70071,7 +70091,7 @@
         <v>36</v>
       </c>
       <c r="G105" s="1" t="s">
-        <v>3467</v>
+        <v>3466</v>
       </c>
       <c r="H105" s="1" t="s">
         <v>1659</v>
@@ -70162,7 +70182,7 @@
         <v>2598</v>
       </c>
       <c r="B109" s="1" t="s">
-        <v>3382</v>
+        <v>3381</v>
       </c>
       <c r="C109" s="1" t="s">
         <v>292</v>
@@ -70248,13 +70268,13 @@
         <v>2643</v>
       </c>
       <c r="B112" s="1" t="s">
-        <v>3381</v>
+        <v>3380</v>
       </c>
       <c r="C112" s="1" t="s">
         <v>543</v>
       </c>
       <c r="D112" s="1" t="s">
-        <v>3266</v>
+        <v>3265</v>
       </c>
       <c r="E112" s="1" t="s">
         <v>544</v>
@@ -70278,10 +70298,10 @@
         <v>2712</v>
       </c>
       <c r="B113" s="1" t="s">
-        <v>3380</v>
+        <v>3379</v>
       </c>
       <c r="C113" s="1" t="s">
-        <v>3266</v>
+        <v>3265</v>
       </c>
       <c r="D113" s="1" t="s">
         <v>542</v>
@@ -70308,10 +70328,10 @@
         <v>2642</v>
       </c>
       <c r="B114" s="1" t="s">
-        <v>3379</v>
+        <v>3378</v>
       </c>
       <c r="C114" s="1" t="s">
-        <v>3266</v>
+        <v>3265</v>
       </c>
       <c r="D114" s="1" t="s">
         <v>544</v>
@@ -70338,7 +70358,7 @@
         <v>2711</v>
       </c>
       <c r="B115" s="1" t="s">
-        <v>3378</v>
+        <v>3377</v>
       </c>
       <c r="C115" s="1" t="s">
         <v>544</v>
@@ -70347,7 +70367,7 @@
         <v>542</v>
       </c>
       <c r="E115" s="1" t="s">
-        <v>3266</v>
+        <v>3265</v>
       </c>
       <c r="F115" s="1" t="s">
         <v>37</v>
@@ -70377,7 +70397,7 @@
         <v>1094</v>
       </c>
       <c r="E116" s="1" t="s">
-        <v>3265</v>
+        <v>3264</v>
       </c>
       <c r="F116" s="1" t="s">
         <v>35</v>
@@ -70398,7 +70418,7 @@
         <v>2709</v>
       </c>
       <c r="B117" s="1" t="s">
-        <v>3377</v>
+        <v>3376</v>
       </c>
       <c r="C117" s="1" t="s">
         <v>1617</v>
@@ -70428,7 +70448,7 @@
         <v>2597</v>
       </c>
       <c r="B118" s="1" t="s">
-        <v>3376</v>
+        <v>3375</v>
       </c>
       <c r="C118" s="1" t="s">
         <v>1616</v>
@@ -70473,7 +70493,7 @@
         <v>37</v>
       </c>
       <c r="G119" s="1" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="H119" s="1" t="s">
         <v>1659</v>
@@ -70553,7 +70573,7 @@
         <v>2237</v>
       </c>
       <c r="C122" s="1" t="s">
-        <v>3329</v>
+        <v>3328</v>
       </c>
       <c r="D122" s="1" t="s">
         <v>1087</v>
@@ -70580,13 +70600,13 @@
         <v>2638</v>
       </c>
       <c r="B123" s="1" t="s">
-        <v>3375</v>
+        <v>3374</v>
       </c>
       <c r="C123" s="1" t="s">
-        <v>3328</v>
+        <v>3327</v>
       </c>
       <c r="D123" s="1" t="s">
-        <v>3299</v>
+        <v>3298</v>
       </c>
       <c r="E123" s="1" t="s">
         <v>363</v>
@@ -70643,7 +70663,7 @@
         <v>2234</v>
       </c>
       <c r="C125" s="1" t="s">
-        <v>3416</v>
+        <v>3415</v>
       </c>
       <c r="D125" s="1" t="s">
         <v>1084</v>
@@ -70706,10 +70726,10 @@
         <v>1605</v>
       </c>
       <c r="D127" s="1" t="s">
-        <v>3298</v>
+        <v>3297</v>
       </c>
       <c r="E127" s="1" t="s">
-        <v>3264</v>
+        <v>3263</v>
       </c>
       <c r="F127" s="1" t="s">
         <v>37</v>
@@ -70729,13 +70749,13 @@
         <v>2230</v>
       </c>
       <c r="C128" s="1" t="s">
-        <v>3327</v>
+        <v>3326</v>
       </c>
       <c r="D128" s="1" t="s">
-        <v>3297</v>
+        <v>3296</v>
       </c>
       <c r="E128" s="1" t="s">
-        <v>3263</v>
+        <v>3262</v>
       </c>
       <c r="F128" s="1" t="s">
         <v>35</v>
@@ -70758,7 +70778,7 @@
         <v>1603</v>
       </c>
       <c r="D129" s="1" t="s">
-        <v>3296</v>
+        <v>3295</v>
       </c>
       <c r="E129" s="1" t="s">
         <v>526</v>
@@ -70971,7 +70991,7 @@
         <v>1076</v>
       </c>
       <c r="E136" s="1" t="s">
-        <v>3262</v>
+        <v>3261</v>
       </c>
       <c r="F136" s="1" t="s">
         <v>35</v>
@@ -71047,13 +71067,13 @@
         <v>2220</v>
       </c>
       <c r="C139" s="1" t="s">
-        <v>3326</v>
+        <v>3325</v>
       </c>
       <c r="D139" s="1" t="s">
         <v>1074</v>
       </c>
       <c r="E139" s="1" t="s">
-        <v>3261</v>
+        <v>3260</v>
       </c>
       <c r="F139" s="1" t="s">
         <v>36</v>
@@ -71074,7 +71094,7 @@
         <v>2696</v>
       </c>
       <c r="B140" s="1" t="s">
-        <v>3374</v>
+        <v>3373</v>
       </c>
       <c r="C140" s="1" t="s">
         <v>1596</v>
@@ -71083,7 +71103,7 @@
         <v>1073</v>
       </c>
       <c r="E140" s="1" t="s">
-        <v>3260</v>
+        <v>3259</v>
       </c>
       <c r="F140" s="1" t="s">
         <v>35</v>
@@ -71106,7 +71126,7 @@
         <v>1595</v>
       </c>
       <c r="D141" s="1" t="s">
-        <v>3295</v>
+        <v>3294</v>
       </c>
       <c r="E141" s="1" t="s">
         <v>516</v>
@@ -71130,13 +71150,13 @@
         <v>2593</v>
       </c>
       <c r="B142" s="1" t="s">
-        <v>3373</v>
+        <v>3372</v>
       </c>
       <c r="C142" s="1" t="s">
         <v>1594</v>
       </c>
       <c r="D142" s="1" t="s">
-        <v>3294</v>
+        <v>3293</v>
       </c>
       <c r="E142" s="1" t="s">
         <v>444</v>
@@ -71220,16 +71240,16 @@
         <v>2694</v>
       </c>
       <c r="B145" s="1" t="s">
-        <v>3372</v>
+        <v>3371</v>
       </c>
       <c r="C145" s="1" t="s">
-        <v>3325</v>
+        <v>3324</v>
       </c>
       <c r="D145" s="1" t="s">
-        <v>3293</v>
+        <v>3292</v>
       </c>
       <c r="E145" s="1" t="s">
-        <v>3259</v>
+        <v>3258</v>
       </c>
       <c r="F145" s="1" t="s">
         <v>35</v>
@@ -71250,10 +71270,10 @@
         <v>2693</v>
       </c>
       <c r="B146" s="1" t="s">
-        <v>3371</v>
+        <v>3370</v>
       </c>
       <c r="C146" s="1" t="s">
-        <v>3324</v>
+        <v>3323</v>
       </c>
       <c r="D146" s="1" t="s">
         <v>1007</v>
@@ -71265,7 +71285,7 @@
         <v>36</v>
       </c>
       <c r="G146" s="1" t="s">
-        <v>3494</v>
+        <v>3493</v>
       </c>
       <c r="H146" s="1" t="s">
         <v>1659</v>
@@ -71282,7 +71302,7 @@
         <v>2692</v>
       </c>
       <c r="B147" s="1" t="s">
-        <v>3420</v>
+        <v>3419</v>
       </c>
       <c r="C147" s="1" t="s">
         <v>1589</v>
@@ -71308,7 +71328,7 @@
         <v>2691</v>
       </c>
       <c r="B148" s="1" t="s">
-        <v>3370</v>
+        <v>3369</v>
       </c>
       <c r="C148" s="1" t="s">
         <v>1588</v>
@@ -71347,7 +71367,7 @@
         <v>1065</v>
       </c>
       <c r="E149" s="1" t="s">
-        <v>3402</v>
+        <v>3401</v>
       </c>
       <c r="F149" s="1" t="s">
         <v>35</v>
@@ -71371,7 +71391,7 @@
         <v>2209</v>
       </c>
       <c r="C150" s="1" t="s">
-        <v>3323</v>
+        <v>3322</v>
       </c>
       <c r="D150" s="1" t="s">
         <v>1064</v>
@@ -71530,7 +71550,7 @@
         <v>2685</v>
       </c>
       <c r="B156" s="1" t="s">
-        <v>3369</v>
+        <v>3368</v>
       </c>
       <c r="C156" s="1" t="s">
         <v>1517</v>
@@ -71545,7 +71565,7 @@
         <v>35</v>
       </c>
       <c r="G156" s="1" t="s">
-        <v>3233</v>
+        <v>3232</v>
       </c>
       <c r="H156" s="1" t="s">
         <v>1659</v>
@@ -71614,7 +71634,7 @@
         <v>2682</v>
       </c>
       <c r="B159" s="1" t="s">
-        <v>3368</v>
+        <v>3367</v>
       </c>
       <c r="C159" s="1" t="s">
         <v>1514</v>
@@ -71666,7 +71686,7 @@
         <v>2680</v>
       </c>
       <c r="B161" s="1" t="s">
-        <v>3367</v>
+        <v>3366</v>
       </c>
       <c r="C161" s="1" t="s">
         <v>1513</v>
@@ -71687,7 +71707,7 @@
       <c r="I161" s="1"/>
       <c r="J161" s="1"/>
     </row>
-    <row r="162" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A162" s="1" t="s">
         <v>2679</v>
       </c>
@@ -71706,7 +71726,9 @@
       <c r="F162" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="G162" s="1"/>
+      <c r="G162" s="1" t="s">
+        <v>3497</v>
+      </c>
       <c r="H162" s="1" t="s">
         <v>1659</v>
       </c>
@@ -71815,7 +71837,7 @@
         <v>36</v>
       </c>
       <c r="G166" s="1" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="H166" s="1" t="s">
         <v>1659</v>
@@ -71858,7 +71880,7 @@
         <v>2673</v>
       </c>
       <c r="B168" s="1" t="s">
-        <v>3366</v>
+        <v>3365</v>
       </c>
       <c r="C168" s="1" t="s">
         <v>1576</v>
@@ -71976,7 +71998,9 @@
       <c r="F172" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="G172" s="1"/>
+      <c r="G172" s="1" t="s">
+        <v>3497</v>
+      </c>
       <c r="H172" s="1" t="s">
         <v>1659</v>
       </c>
@@ -72003,7 +72027,7 @@
         <v>36</v>
       </c>
       <c r="G173" s="1" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="H173" s="1" t="s">
         <v>1659</v>
@@ -72019,10 +72043,10 @@
         <v>2184</v>
       </c>
       <c r="C174" s="1" t="s">
-        <v>3258</v>
+        <v>3257</v>
       </c>
       <c r="D174" s="1" t="s">
-        <v>3409</v>
+        <v>3408</v>
       </c>
       <c r="E174" s="1" t="s">
         <v>488</v>
@@ -72048,7 +72072,7 @@
         <v>1046</v>
       </c>
       <c r="D175" s="1" t="s">
-        <v>3258</v>
+        <v>3257</v>
       </c>
       <c r="E175" s="1" t="s">
         <v>486</v>
@@ -72071,13 +72095,13 @@
         <v>2182</v>
       </c>
       <c r="C176" s="1" t="s">
-        <v>3415</v>
+        <v>3414</v>
       </c>
       <c r="D176" s="1" t="s">
         <v>1047</v>
       </c>
       <c r="E176" s="1" t="s">
-        <v>3258</v>
+        <v>3257</v>
       </c>
       <c r="F176" s="1" t="s">
         <v>36</v>
@@ -72097,7 +72121,7 @@
         <v>2181</v>
       </c>
       <c r="C177" s="1" t="s">
-        <v>3258</v>
+        <v>3257</v>
       </c>
       <c r="D177" s="1" t="s">
         <v>1046</v>
@@ -72152,7 +72176,7 @@
         <v>479</v>
       </c>
       <c r="D179" s="1" t="s">
-        <v>3408</v>
+        <v>3407</v>
       </c>
       <c r="E179" s="1" t="s">
         <v>478</v>
@@ -73095,10 +73119,10 @@
         <v>2142</v>
       </c>
       <c r="C215" s="1" t="s">
-        <v>3322</v>
+        <v>3321</v>
       </c>
       <c r="D215" s="1" t="s">
-        <v>3292</v>
+        <v>3291</v>
       </c>
       <c r="E215" s="1" t="s">
         <v>462</v>
@@ -73118,7 +73142,7 @@
         <v>3084</v>
       </c>
       <c r="B216" s="1" t="s">
-        <v>3365</v>
+        <v>3364</v>
       </c>
       <c r="C216" s="1" t="s">
         <v>1491</v>
@@ -73163,7 +73187,7 @@
         <v>36</v>
       </c>
       <c r="G217" s="1" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="H217" s="1" t="s">
         <v>1659</v>
@@ -73186,7 +73210,7 @@
         <v>1561</v>
       </c>
       <c r="D218" s="1" t="s">
-        <v>3291</v>
+        <v>3290</v>
       </c>
       <c r="E218" s="1" t="s">
         <v>460</v>
@@ -73225,7 +73249,7 @@
         <v>35</v>
       </c>
       <c r="G219" s="1" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="H219" s="1" t="s">
         <v>1659</v>
@@ -73271,7 +73295,7 @@
         <v>2136</v>
       </c>
       <c r="C221" s="1" t="s">
-        <v>3321</v>
+        <v>3320</v>
       </c>
       <c r="D221" s="1" t="s">
         <v>1029</v>
@@ -73358,22 +73382,22 @@
         <v>3076</v>
       </c>
       <c r="B224" s="1" t="s">
-        <v>3364</v>
+        <v>3363</v>
       </c>
       <c r="C224" s="1" t="s">
-        <v>3320</v>
+        <v>3319</v>
       </c>
       <c r="D224" s="1" t="s">
-        <v>3290</v>
+        <v>3289</v>
       </c>
       <c r="E224" s="1" t="s">
-        <v>3257</v>
+        <v>3256</v>
       </c>
       <c r="F224" s="1" t="s">
         <v>36</v>
       </c>
       <c r="G224" s="1" t="s">
-        <v>3233</v>
+        <v>3232</v>
       </c>
       <c r="H224" s="1" t="s">
         <v>1659</v>
@@ -73491,7 +73515,7 @@
         <v>37</v>
       </c>
       <c r="G228" s="1" t="s">
-        <v>3465</v>
+        <v>3464</v>
       </c>
       <c r="H228" s="1" t="s">
         <v>1659</v>
@@ -73547,7 +73571,7 @@
         <v>35</v>
       </c>
       <c r="G230" s="1" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="H230" s="1" t="s">
         <v>1659</v>
@@ -73659,7 +73683,7 @@
         <v>966</v>
       </c>
       <c r="E234" s="1" t="s">
-        <v>3256</v>
+        <v>3255</v>
       </c>
       <c r="F234" s="1" t="s">
         <v>37</v>
@@ -73683,13 +73707,13 @@
         <v>2120</v>
       </c>
       <c r="C235" s="1" t="s">
-        <v>3319</v>
+        <v>3318</v>
       </c>
       <c r="D235" s="1" t="s">
         <v>1014</v>
       </c>
       <c r="E235" s="1" t="s">
-        <v>3255</v>
+        <v>3254</v>
       </c>
       <c r="F235" s="1" t="s">
         <v>37</v>
@@ -73751,7 +73775,7 @@
         <v>35</v>
       </c>
       <c r="G237" s="1" t="s">
-        <v>3468</v>
+        <v>3467</v>
       </c>
       <c r="H237" s="1" t="s">
         <v>1659</v>
@@ -73779,7 +73803,7 @@
         <v>35</v>
       </c>
       <c r="G238" s="1" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="H238" s="1" t="s">
         <v>1659</v>
@@ -73811,7 +73835,7 @@
         <v>35</v>
       </c>
       <c r="G239" s="1" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="H239" s="1" t="s">
         <v>1659</v>
@@ -73824,7 +73848,7 @@
         <v>3059</v>
       </c>
       <c r="B240" s="1" t="s">
-        <v>3363</v>
+        <v>3362</v>
       </c>
       <c r="C240" s="1" t="s">
         <v>1490</v>
@@ -73839,7 +73863,7 @@
         <v>35</v>
       </c>
       <c r="G240" s="1" t="s">
-        <v>3233</v>
+        <v>3232</v>
       </c>
       <c r="H240" s="1" t="s">
         <v>1659</v>
@@ -73852,16 +73876,16 @@
         <v>3058</v>
       </c>
       <c r="B241" s="1" t="s">
-        <v>3362</v>
+        <v>3361</v>
       </c>
       <c r="C241" s="1" t="s">
         <v>1033</v>
       </c>
       <c r="D241" s="1" t="s">
-        <v>3289</v>
+        <v>3288</v>
       </c>
       <c r="E241" s="1" t="s">
-        <v>3254</v>
+        <v>3253</v>
       </c>
       <c r="F241" s="1" t="s">
         <v>37</v>
@@ -73949,7 +73973,7 @@
         <v>35</v>
       </c>
       <c r="G244" s="1" t="s">
-        <v>3487</v>
+        <v>3486</v>
       </c>
       <c r="H244" s="1" t="s">
         <v>1659</v>
@@ -74037,7 +74061,7 @@
         <v>35</v>
       </c>
       <c r="G247" s="1" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="H247" s="1" t="s">
         <v>1659</v>
@@ -74065,7 +74089,7 @@
         <v>36</v>
       </c>
       <c r="G248" s="1" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="H248" s="1" t="s">
         <v>1659</v>
@@ -74093,7 +74117,7 @@
         <v>35</v>
       </c>
       <c r="G249" s="1" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="H249" s="1" t="s">
         <v>1659</v>
@@ -74125,7 +74149,7 @@
         <v>35</v>
       </c>
       <c r="G250" s="1" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="H250" s="1" t="s">
         <v>1659</v>
@@ -74141,7 +74165,7 @@
         <v>2271</v>
       </c>
       <c r="C251" s="1" t="s">
-        <v>3330</v>
+        <v>3329</v>
       </c>
       <c r="D251" s="1" t="s">
         <v>1104</v>
@@ -74179,7 +74203,7 @@
         <v>37</v>
       </c>
       <c r="G252" s="1" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="H252" s="1" t="s">
         <v>1659</v>
@@ -74207,7 +74231,7 @@
         <v>36</v>
       </c>
       <c r="G253" s="1" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="H253" s="1" t="s">
         <v>1659</v>
@@ -74235,7 +74259,7 @@
         <v>37</v>
       </c>
       <c r="G254" s="1" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="H254" s="1" t="s">
         <v>1659</v>
@@ -74263,7 +74287,7 @@
         <v>37</v>
       </c>
       <c r="G255" s="1" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="H255" s="1" t="s">
         <v>1659</v>
@@ -74291,7 +74315,7 @@
         <v>35</v>
       </c>
       <c r="G256" s="1" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="H256" s="1" t="s">
         <v>1659</v>
@@ -74323,7 +74347,7 @@
         <v>37</v>
       </c>
       <c r="G257" s="1" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="H257" s="1" t="s">
         <v>1659</v>
@@ -74351,7 +74375,7 @@
         <v>35</v>
       </c>
       <c r="G258" s="1" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="H258" s="1" t="s">
         <v>1659</v>
@@ -74379,7 +74403,7 @@
         <v>36</v>
       </c>
       <c r="G259" s="1" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="H259" s="1" t="s">
         <v>1659</v>
@@ -74392,7 +74416,7 @@
         <v>3040</v>
       </c>
       <c r="B260" s="1" t="s">
-        <v>3361</v>
+        <v>3360</v>
       </c>
       <c r="C260" s="1" t="s">
         <v>1518</v>
@@ -74401,13 +74425,13 @@
         <v>988</v>
       </c>
       <c r="E260" s="1" t="s">
-        <v>3253</v>
+        <v>3252</v>
       </c>
       <c r="F260" s="1" t="s">
         <v>37</v>
       </c>
       <c r="G260" s="1" t="s">
-        <v>3233</v>
+        <v>3232</v>
       </c>
       <c r="H260" s="1" t="s">
         <v>1659</v>
@@ -74420,7 +74444,7 @@
         <v>3039</v>
       </c>
       <c r="B261" s="1" t="s">
-        <v>3360</v>
+        <v>3359</v>
       </c>
       <c r="C261" s="1" t="s">
         <v>1517</v>
@@ -74435,7 +74459,7 @@
         <v>35</v>
       </c>
       <c r="G261" s="1" t="s">
-        <v>3233</v>
+        <v>3232</v>
       </c>
       <c r="H261" s="1" t="s">
         <v>1659</v>
@@ -74463,7 +74487,7 @@
         <v>36</v>
       </c>
       <c r="G262" s="1" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="H262" s="1" t="s">
         <v>1659</v>
@@ -74491,7 +74515,7 @@
         <v>36</v>
       </c>
       <c r="G263" s="1" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="H263" s="1" t="s">
         <v>1659</v>
@@ -74504,7 +74528,7 @@
         <v>3036</v>
       </c>
       <c r="B264" s="1" t="s">
-        <v>3359</v>
+        <v>3358</v>
       </c>
       <c r="C264" s="1" t="s">
         <v>1513</v>
@@ -74545,7 +74569,7 @@
         <v>37</v>
       </c>
       <c r="G265" s="1" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="H265" s="1" t="s">
         <v>1659</v>
@@ -74573,7 +74597,7 @@
         <v>36</v>
       </c>
       <c r="G266" s="1" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="H266" s="1" t="s">
         <v>1659</v>
@@ -74601,7 +74625,7 @@
         <v>35</v>
       </c>
       <c r="G267" s="1" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="H267" s="1" t="s">
         <v>1659</v>
@@ -74629,7 +74653,7 @@
         <v>37</v>
       </c>
       <c r="G268" s="1" t="s">
-        <v>3465</v>
+        <v>3464</v>
       </c>
       <c r="H268" s="1" t="s">
         <v>1659</v>
@@ -74661,7 +74685,7 @@
         <v>35</v>
       </c>
       <c r="G269" s="1" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="H269" s="1" t="s">
         <v>1659</v>
@@ -74689,7 +74713,7 @@
         <v>35</v>
       </c>
       <c r="G270" s="1" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="H270" s="1" t="s">
         <v>1659</v>
@@ -74717,7 +74741,7 @@
         <v>37</v>
       </c>
       <c r="G271" s="1" t="s">
-        <v>3469</v>
+        <v>3468</v>
       </c>
       <c r="H271" s="1" t="s">
         <v>1659</v>
@@ -74745,7 +74769,7 @@
         <v>36</v>
       </c>
       <c r="G272" s="1" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="H272" s="1" t="s">
         <v>1659</v>
@@ -74823,7 +74847,7 @@
         <v>36</v>
       </c>
       <c r="G275" s="1" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="H275" s="1" t="s">
         <v>1659</v>
@@ -74851,7 +74875,7 @@
         <v>36</v>
       </c>
       <c r="G276" s="1" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="H276" s="1" t="s">
         <v>1659</v>
@@ -74883,7 +74907,7 @@
         <v>36</v>
       </c>
       <c r="G277" s="1" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="H277" s="1" t="s">
         <v>1659</v>
@@ -74967,7 +74991,7 @@
         <v>37</v>
       </c>
       <c r="G280" s="1" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="H280" s="1" t="s">
         <v>1659</v>
@@ -74995,7 +75019,7 @@
         <v>37</v>
       </c>
       <c r="G281" s="1" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="H281" s="1" t="s">
         <v>1659</v>
@@ -75023,7 +75047,7 @@
         <v>36</v>
       </c>
       <c r="G282" s="1" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="H282" s="1" t="s">
         <v>1659</v>
@@ -75055,7 +75079,7 @@
         <v>37</v>
       </c>
       <c r="G283" s="1" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="H283" s="1" t="s">
         <v>1659</v>
@@ -75132,22 +75156,22 @@
         <v>3015</v>
       </c>
       <c r="B286" s="1" t="s">
-        <v>3358</v>
+        <v>3357</v>
       </c>
       <c r="C286" s="1" t="s">
-        <v>3318</v>
+        <v>3317</v>
       </c>
       <c r="D286" s="1" t="s">
-        <v>3288</v>
+        <v>3287</v>
       </c>
       <c r="E286" s="1" t="s">
-        <v>3252</v>
+        <v>3251</v>
       </c>
       <c r="F286" s="1" t="s">
         <v>37</v>
       </c>
       <c r="G286" s="1" t="s">
-        <v>3233</v>
+        <v>3232</v>
       </c>
       <c r="H286" s="1" t="s">
         <v>1659</v>
@@ -75179,7 +75203,7 @@
         <v>35</v>
       </c>
       <c r="G287" s="1" t="s">
-        <v>3470</v>
+        <v>3469</v>
       </c>
       <c r="H287" s="1" t="s">
         <v>1659</v>
@@ -75207,7 +75231,7 @@
         <v>36</v>
       </c>
       <c r="G288" s="1" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="H288" s="1" t="s">
         <v>1659</v>
@@ -75235,7 +75259,7 @@
         <v>37</v>
       </c>
       <c r="G289" s="1" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="H289" s="1" t="s">
         <v>1659</v>
@@ -75267,7 +75291,7 @@
         <v>36</v>
       </c>
       <c r="G290" s="1" t="s">
-        <v>3471</v>
+        <v>3470</v>
       </c>
       <c r="H290" s="1" t="s">
         <v>1659</v>
@@ -75275,7 +75299,7 @@
       <c r="I290" s="1"/>
       <c r="J290" s="1"/>
     </row>
-    <row r="291" spans="1:10" ht="105" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A291" s="1" t="s">
         <v>3009</v>
       </c>
@@ -75292,10 +75316,10 @@
         <v>384</v>
       </c>
       <c r="F291" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G291" s="1" t="s">
-        <v>3495</v>
+        <v>3497</v>
       </c>
       <c r="H291" s="1" t="s">
         <v>1659</v>
@@ -75327,7 +75351,7 @@
         <v>36</v>
       </c>
       <c r="G292" s="1" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="H292" s="1" t="s">
         <v>1659</v>
@@ -75340,22 +75364,22 @@
         <v>3007</v>
       </c>
       <c r="B293" s="1" t="s">
-        <v>3357</v>
+        <v>3356</v>
       </c>
       <c r="C293" s="1" t="s">
-        <v>3317</v>
+        <v>3316</v>
       </c>
       <c r="D293" s="1" t="s">
-        <v>3287</v>
+        <v>3286</v>
       </c>
       <c r="E293" s="1" t="s">
-        <v>3251</v>
+        <v>3250</v>
       </c>
       <c r="F293" s="1" t="s">
         <v>37</v>
       </c>
       <c r="G293" s="1" t="s">
-        <v>3233</v>
+        <v>3232</v>
       </c>
       <c r="H293" s="1" t="s">
         <v>1659</v>
@@ -75413,7 +75437,7 @@
         <v>37</v>
       </c>
       <c r="G295" s="1" t="s">
-        <v>3472</v>
+        <v>3471</v>
       </c>
       <c r="H295" s="1" t="s">
         <v>1659</v>
@@ -75475,7 +75499,7 @@
         <v>35</v>
       </c>
       <c r="G297" s="1" t="s">
-        <v>3473</v>
+        <v>3472</v>
       </c>
       <c r="H297" s="1" t="s">
         <v>1659</v>
@@ -75507,7 +75531,7 @@
         <v>37</v>
       </c>
       <c r="G298" s="1" t="s">
-        <v>3474</v>
+        <v>3473</v>
       </c>
       <c r="H298" s="1" t="s">
         <v>1659</v>
@@ -75565,7 +75589,7 @@
         <v>37</v>
       </c>
       <c r="G300" s="1" t="s">
-        <v>3475</v>
+        <v>3474</v>
       </c>
       <c r="H300" s="1" t="s">
         <v>1659</v>
@@ -75683,7 +75707,7 @@
         <v>37</v>
       </c>
       <c r="G304" s="1" t="s">
-        <v>3476</v>
+        <v>3475</v>
       </c>
       <c r="H304" s="1" t="s">
         <v>1659</v>
@@ -75711,7 +75735,7 @@
         <v>35</v>
       </c>
       <c r="G305" s="1" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="H305" s="1" t="s">
         <v>1659</v>
@@ -75724,16 +75748,16 @@
         <v>2994</v>
       </c>
       <c r="B306" s="1" t="s">
-        <v>3356</v>
+        <v>3355</v>
       </c>
       <c r="C306" s="1" t="s">
-        <v>3316</v>
+        <v>3315</v>
       </c>
       <c r="D306" s="1" t="s">
-        <v>3286</v>
+        <v>3285</v>
       </c>
       <c r="E306" s="1" t="s">
-        <v>3401</v>
+        <v>3400</v>
       </c>
       <c r="F306" s="1" t="s">
         <v>35</v>
@@ -75799,7 +75823,7 @@
         <v>36</v>
       </c>
       <c r="G308" s="1" t="s">
-        <v>3496</v>
+        <v>3494</v>
       </c>
       <c r="H308" s="1" t="s">
         <v>1659</v>
@@ -75831,7 +75855,7 @@
         <v>37</v>
       </c>
       <c r="G309" s="1" t="s">
-        <v>3485</v>
+        <v>3484</v>
       </c>
       <c r="H309" s="1" t="s">
         <v>1659</v>
@@ -75904,13 +75928,13 @@
         <v>2988</v>
       </c>
       <c r="B312" s="1" t="s">
-        <v>3355</v>
+        <v>3354</v>
       </c>
       <c r="C312" s="1" t="s">
-        <v>3315</v>
+        <v>3314</v>
       </c>
       <c r="D312" s="1" t="s">
-        <v>3285</v>
+        <v>3284</v>
       </c>
       <c r="E312" s="1" t="s">
         <v>363</v>
@@ -75979,7 +76003,7 @@
         <v>37</v>
       </c>
       <c r="G314" s="1" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="H314" s="1" t="s">
         <v>1659</v>
@@ -76037,7 +76061,7 @@
         <v>36</v>
       </c>
       <c r="G316" s="1" t="s">
-        <v>3477</v>
+        <v>3476</v>
       </c>
       <c r="H316" s="1" t="s">
         <v>1659</v>
@@ -76050,16 +76074,16 @@
         <v>2983</v>
       </c>
       <c r="B317" s="1" t="s">
-        <v>3354</v>
+        <v>3353</v>
       </c>
       <c r="C317" s="1" t="s">
-        <v>3314</v>
+        <v>3313</v>
       </c>
       <c r="D317" s="1" t="s">
-        <v>3284</v>
+        <v>3283</v>
       </c>
       <c r="E317" s="1" t="s">
-        <v>3250</v>
+        <v>3249</v>
       </c>
       <c r="F317" s="1" t="s">
         <v>36</v>
@@ -76155,7 +76179,7 @@
         <v>37</v>
       </c>
       <c r="G320" s="1" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="H320" s="1" t="s">
         <v>1659</v>
@@ -76213,7 +76237,7 @@
         <v>36</v>
       </c>
       <c r="G322" s="1" t="s">
-        <v>3478</v>
+        <v>3477</v>
       </c>
       <c r="H322" s="1" t="s">
         <v>1659</v>
@@ -76290,7 +76314,7 @@
         <v>2975</v>
       </c>
       <c r="B325" s="1" t="s">
-        <v>3353</v>
+        <v>3352</v>
       </c>
       <c r="C325" s="1" t="s">
         <v>1453</v>
@@ -76447,7 +76471,7 @@
         <v>37</v>
       </c>
       <c r="G330" s="1" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="H330" s="1" t="s">
         <v>1659</v>
@@ -76535,7 +76559,7 @@
         <v>37</v>
       </c>
       <c r="G333" s="1" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="H333" s="1" t="s">
         <v>1659</v>
@@ -76593,7 +76617,7 @@
         <v>37</v>
       </c>
       <c r="G335" s="1" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="H335" s="1" t="s">
         <v>1659</v>
@@ -76625,7 +76649,7 @@
         <v>36</v>
       </c>
       <c r="G336" s="1" t="s">
-        <v>3462</v>
+        <v>3461</v>
       </c>
       <c r="H336" s="1" t="s">
         <v>1659</v>
@@ -76759,10 +76783,10 @@
     </row>
     <row r="341" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A341" s="1" t="s">
-        <v>3444</v>
+        <v>3443</v>
       </c>
       <c r="B341" s="1" t="s">
-        <v>3419</v>
+        <v>3418</v>
       </c>
       <c r="C341" s="1"/>
       <c r="D341" s="1"/>
@@ -76780,7 +76804,7 @@
         <v>2962</v>
       </c>
       <c r="B342" s="1" t="s">
-        <v>3352</v>
+        <v>3351</v>
       </c>
       <c r="C342" s="1" t="s">
         <v>1404</v>
@@ -76872,7 +76896,7 @@
         <v>1401</v>
       </c>
       <c r="D345" s="1" t="s">
-        <v>3283</v>
+        <v>3282</v>
       </c>
       <c r="E345" s="1" t="s">
         <v>283</v>
@@ -77076,16 +77100,16 @@
         <v>2952</v>
       </c>
       <c r="B352" s="1" t="s">
-        <v>3351</v>
+        <v>3350</v>
       </c>
       <c r="C352" s="1" t="s">
         <v>1396</v>
       </c>
       <c r="D352" s="1" t="s">
-        <v>3282</v>
+        <v>3281</v>
       </c>
       <c r="E352" s="1" t="s">
-        <v>3249</v>
+        <v>3248</v>
       </c>
       <c r="F352" s="1" t="s">
         <v>37</v>
@@ -77112,7 +77136,7 @@
         <v>1395</v>
       </c>
       <c r="D353" s="1" t="s">
-        <v>3281</v>
+        <v>3280</v>
       </c>
       <c r="E353" s="1" t="s">
         <v>277</v>
@@ -77151,7 +77175,7 @@
         <v>37</v>
       </c>
       <c r="G354" s="1" t="s">
-        <v>3479</v>
+        <v>3478</v>
       </c>
       <c r="H354" s="1" t="s">
         <v>1659</v>
@@ -77168,13 +77192,13 @@
         <v>2949</v>
       </c>
       <c r="B355" s="1" t="s">
-        <v>3350</v>
+        <v>3349</v>
       </c>
       <c r="C355" s="1" t="s">
         <v>832</v>
       </c>
       <c r="D355" s="1" t="s">
-        <v>3280</v>
+        <v>3279</v>
       </c>
       <c r="E355" s="1" t="s">
         <v>242</v>
@@ -77183,7 +77207,7 @@
         <v>36</v>
       </c>
       <c r="G355" s="1" t="s">
-        <v>3232</v>
+        <v>3231</v>
       </c>
       <c r="H355" s="1" t="s">
         <v>1659</v>
@@ -77200,16 +77224,16 @@
         <v>2948</v>
       </c>
       <c r="B356" s="1" t="s">
-        <v>3349</v>
+        <v>3348</v>
       </c>
       <c r="C356" s="1" t="s">
-        <v>3313</v>
+        <v>3312</v>
       </c>
       <c r="D356" s="1" t="s">
-        <v>3279</v>
+        <v>3278</v>
       </c>
       <c r="E356" s="1" t="s">
-        <v>3248</v>
+        <v>3247</v>
       </c>
       <c r="F356" s="1" t="s">
         <v>37</v>
@@ -77479,7 +77503,7 @@
         <v>854</v>
       </c>
       <c r="E365" s="1" t="s">
-        <v>3247</v>
+        <v>3246</v>
       </c>
       <c r="F365" s="1" t="s">
         <v>35</v>
@@ -77509,7 +77533,7 @@
         <v>853</v>
       </c>
       <c r="E366" s="1" t="s">
-        <v>3246</v>
+        <v>3245</v>
       </c>
       <c r="F366" s="1" t="s">
         <v>35</v>
@@ -77650,16 +77674,16 @@
         <v>2933</v>
       </c>
       <c r="B371" s="1" t="s">
-        <v>3348</v>
+        <v>3347</v>
       </c>
       <c r="C371" s="1" t="s">
-        <v>3312</v>
+        <v>3311</v>
       </c>
       <c r="D371" s="1" t="s">
         <v>1389</v>
       </c>
       <c r="E371" s="1" t="s">
-        <v>3245</v>
+        <v>3244</v>
       </c>
       <c r="F371" s="1" t="s">
         <v>37</v>
@@ -77890,16 +77914,16 @@
         <v>2925</v>
       </c>
       <c r="B379" s="1" t="s">
-        <v>3347</v>
+        <v>3346</v>
       </c>
       <c r="C379" s="1" t="s">
-        <v>3311</v>
+        <v>3310</v>
       </c>
       <c r="D379" s="1" t="s">
-        <v>3278</v>
+        <v>3277</v>
       </c>
       <c r="E379" s="1" t="s">
-        <v>3244</v>
+        <v>3243</v>
       </c>
       <c r="F379" s="1" t="s">
         <v>35</v>
@@ -77915,27 +77939,27 @@
         <v>2926</v>
       </c>
     </row>
-    <row r="380" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="380" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A380" s="1" t="s">
         <v>2924</v>
       </c>
       <c r="B380" s="1" t="s">
-        <v>3346</v>
+        <v>3345</v>
       </c>
       <c r="C380" s="1" t="s">
-        <v>3310</v>
+        <v>3309</v>
       </c>
       <c r="D380" s="1" t="s">
-        <v>3277</v>
+        <v>3276</v>
       </c>
       <c r="E380" s="1" t="s">
-        <v>3243</v>
+        <v>3242</v>
       </c>
       <c r="F380" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G380" s="1" t="s">
-        <v>3231</v>
+        <v>3497</v>
       </c>
       <c r="H380" s="1" t="s">
         <v>1659</v>
@@ -77979,10 +78003,10 @@
     </row>
     <row r="382" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A382" s="1" t="s">
-        <v>3443</v>
+        <v>3442</v>
       </c>
       <c r="B382" s="1" t="s">
-        <v>3418</v>
+        <v>3417</v>
       </c>
       <c r="C382" s="1"/>
       <c r="D382" s="1"/>
@@ -78726,7 +78750,7 @@
         <v>1317</v>
       </c>
       <c r="D407" s="1" t="s">
-        <v>3407</v>
+        <v>3406</v>
       </c>
       <c r="E407" s="1" t="s">
         <v>193</v>
@@ -78753,13 +78777,13 @@
         <v>1855</v>
       </c>
       <c r="C408" s="1" t="s">
-        <v>3309</v>
+        <v>3308</v>
       </c>
       <c r="D408" s="1" t="s">
         <v>779</v>
       </c>
       <c r="E408" s="1" t="s">
-        <v>3242</v>
+        <v>3241</v>
       </c>
       <c r="F408" s="1" t="s">
         <v>35</v>
@@ -78780,10 +78804,10 @@
         <v>2896</v>
       </c>
       <c r="B409" s="1" t="s">
-        <v>3345</v>
+        <v>3344</v>
       </c>
       <c r="C409" s="1" t="s">
-        <v>3308</v>
+        <v>3307</v>
       </c>
       <c r="D409" s="1" t="s">
         <v>778</v>
@@ -78810,13 +78834,13 @@
         <v>2895</v>
       </c>
       <c r="B410" s="1" t="s">
-        <v>3344</v>
+        <v>3343</v>
       </c>
       <c r="C410" s="1" t="s">
         <v>1314</v>
       </c>
       <c r="D410" s="1" t="s">
-        <v>3406</v>
+        <v>3405</v>
       </c>
       <c r="E410" s="1" t="s">
         <v>190</v>
@@ -79620,7 +79644,7 @@
         <v>2868</v>
       </c>
       <c r="B437" s="1" t="s">
-        <v>3343</v>
+        <v>3342</v>
       </c>
       <c r="C437" s="1" t="s">
         <v>1289</v>
@@ -79629,7 +79653,7 @@
         <v>754</v>
       </c>
       <c r="E437" s="1" t="s">
-        <v>3400</v>
+        <v>3399</v>
       </c>
       <c r="F437" s="1" t="s">
         <v>35</v>
@@ -79980,10 +80004,10 @@
         <v>2856</v>
       </c>
       <c r="B449" s="1" t="s">
-        <v>3342</v>
+        <v>3341</v>
       </c>
       <c r="C449" s="1" t="s">
-        <v>3307</v>
+        <v>3306</v>
       </c>
       <c r="D449" s="1" t="s">
         <v>742</v>
@@ -80025,7 +80049,7 @@
         <v>36</v>
       </c>
       <c r="G450" s="1" t="s">
-        <v>3489</v>
+        <v>3488</v>
       </c>
       <c r="H450" s="1" t="s">
         <v>1659</v>
@@ -80072,16 +80096,16 @@
         <v>2853</v>
       </c>
       <c r="B452" s="1" t="s">
-        <v>3341</v>
+        <v>3340</v>
       </c>
       <c r="C452" s="1" t="s">
-        <v>3306</v>
+        <v>3305</v>
       </c>
       <c r="D452" s="1" t="s">
-        <v>3276</v>
+        <v>3275</v>
       </c>
       <c r="E452" s="1" t="s">
-        <v>3241</v>
+        <v>3240</v>
       </c>
       <c r="F452" s="1" t="s">
         <v>35</v>
@@ -80237,7 +80261,7 @@
         <v>37</v>
       </c>
       <c r="G457" s="1" t="s">
-        <v>3478</v>
+        <v>3477</v>
       </c>
       <c r="H457" s="1" t="s">
         <v>1659</v>
@@ -80251,10 +80275,10 @@
     </row>
     <row r="458" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A458" s="1" t="s">
-        <v>3442</v>
+        <v>3441</v>
       </c>
       <c r="B458" s="1" t="s">
-        <v>3417</v>
+        <v>3416</v>
       </c>
       <c r="C458" s="1"/>
       <c r="D458" s="1"/>
@@ -80377,7 +80401,7 @@
         <v>35</v>
       </c>
       <c r="G462" s="1" t="s">
-        <v>3480</v>
+        <v>3479</v>
       </c>
       <c r="H462" s="1" t="s">
         <v>1659</v>
@@ -80397,13 +80421,13 @@
         <v>1784</v>
       </c>
       <c r="C463" s="1" t="s">
-        <v>3414</v>
+        <v>3413</v>
       </c>
       <c r="D463" s="1" t="s">
-        <v>3405</v>
+        <v>3404</v>
       </c>
       <c r="E463" s="1" t="s">
-        <v>3399</v>
+        <v>3398</v>
       </c>
       <c r="F463" s="1" t="s">
         <v>37</v>
@@ -80459,7 +80483,7 @@
         <v>716</v>
       </c>
       <c r="E465" s="1" t="s">
-        <v>3240</v>
+        <v>3239</v>
       </c>
       <c r="F465" s="1" t="s">
         <v>35</v>
@@ -80483,10 +80507,10 @@
         <v>1781</v>
       </c>
       <c r="C466" s="1" t="s">
-        <v>3413</v>
+        <v>3412</v>
       </c>
       <c r="D466" s="1" t="s">
-        <v>3404</v>
+        <v>3403</v>
       </c>
       <c r="E466" s="1" t="s">
         <v>122</v>
@@ -80540,16 +80564,16 @@
         <v>2838</v>
       </c>
       <c r="B468" s="1" t="s">
-        <v>3340</v>
+        <v>3339</v>
       </c>
       <c r="C468" s="1" t="s">
-        <v>3305</v>
+        <v>3304</v>
       </c>
       <c r="D468" s="1" t="s">
-        <v>3275</v>
+        <v>3274</v>
       </c>
       <c r="E468" s="1" t="s">
-        <v>3239</v>
+        <v>3238</v>
       </c>
       <c r="F468" s="1" t="s">
         <v>37</v>
@@ -80576,7 +80600,7 @@
         <v>1253</v>
       </c>
       <c r="D469" s="1" t="s">
-        <v>3274</v>
+        <v>3273</v>
       </c>
       <c r="E469" s="1" t="s">
         <v>119</v>
@@ -80600,16 +80624,16 @@
         <v>2836</v>
       </c>
       <c r="B470" s="1" t="s">
-        <v>3339</v>
+        <v>3338</v>
       </c>
       <c r="C470" s="1" t="s">
-        <v>3412</v>
+        <v>3411</v>
       </c>
       <c r="D470" s="1" t="s">
-        <v>3398</v>
+        <v>3397</v>
       </c>
       <c r="E470" s="1" t="s">
-        <v>3238</v>
+        <v>3237</v>
       </c>
       <c r="F470" s="1" t="s">
         <v>35</v>
@@ -80633,13 +80657,13 @@
         <v>1776</v>
       </c>
       <c r="C471" s="1" t="s">
-        <v>3412</v>
+        <v>3411</v>
       </c>
       <c r="D471" s="1" t="s">
-        <v>3403</v>
+        <v>3402</v>
       </c>
       <c r="E471" s="1" t="s">
-        <v>3398</v>
+        <v>3397</v>
       </c>
       <c r="F471" s="1" t="s">
         <v>37</v>
@@ -80663,13 +80687,13 @@
         <v>1775</v>
       </c>
       <c r="C472" s="1" t="s">
-        <v>3411</v>
+        <v>3410</v>
       </c>
       <c r="D472" s="1" t="s">
         <v>710</v>
       </c>
       <c r="E472" s="1" t="s">
-        <v>3397</v>
+        <v>3396</v>
       </c>
       <c r="F472" s="1" t="s">
         <v>37</v>
@@ -80810,13 +80834,13 @@
         <v>2829</v>
       </c>
       <c r="B477" s="1" t="s">
-        <v>3338</v>
+        <v>3337</v>
       </c>
       <c r="C477" s="1" t="s">
         <v>115</v>
       </c>
       <c r="D477" s="1" t="s">
-        <v>3273</v>
+        <v>3272</v>
       </c>
       <c r="E477" s="1" t="s">
         <v>111</v>
@@ -80843,13 +80867,13 @@
         <v>1769</v>
       </c>
       <c r="C478" s="1" t="s">
-        <v>3304</v>
+        <v>3303</v>
       </c>
       <c r="D478" s="1" t="s">
         <v>704</v>
       </c>
       <c r="E478" s="1" t="s">
-        <v>3237</v>
+        <v>3236</v>
       </c>
       <c r="F478" s="1" t="s">
         <v>36</v>
@@ -80879,7 +80903,7 @@
         <v>704</v>
       </c>
       <c r="E479" s="1" t="s">
-        <v>3237</v>
+        <v>3236</v>
       </c>
       <c r="F479" s="1" t="s">
         <v>37</v>
@@ -80960,7 +80984,7 @@
         <v>2824</v>
       </c>
       <c r="B482" s="1" t="s">
-        <v>3337</v>
+        <v>3336</v>
       </c>
       <c r="C482" s="1" t="s">
         <v>700</v>
@@ -80990,7 +81014,7 @@
         <v>2823</v>
       </c>
       <c r="B483" s="1" t="s">
-        <v>3336</v>
+        <v>3335</v>
       </c>
       <c r="C483" s="1" t="s">
         <v>1243</v>
@@ -81020,7 +81044,7 @@
         <v>2822</v>
       </c>
       <c r="B484" s="1" t="s">
-        <v>3335</v>
+        <v>3334</v>
       </c>
       <c r="C484" s="1" t="s">
         <v>1242</v>
@@ -81083,10 +81107,10 @@
         <v>1761</v>
       </c>
       <c r="C486" s="1" t="s">
-        <v>3303</v>
+        <v>3302</v>
       </c>
       <c r="D486" s="1" t="s">
-        <v>3272</v>
+        <v>3271</v>
       </c>
       <c r="E486" s="1" t="s">
         <v>103</v>
@@ -81113,13 +81137,13 @@
         <v>1760</v>
       </c>
       <c r="C487" s="1" t="s">
-        <v>3302</v>
+        <v>3301</v>
       </c>
       <c r="D487" s="1" t="s">
         <v>697</v>
       </c>
       <c r="E487" s="1" t="s">
-        <v>3236</v>
+        <v>3235</v>
       </c>
       <c r="F487" s="1" t="s">
         <v>37</v>
@@ -81203,7 +81227,7 @@
         <v>1757</v>
       </c>
       <c r="C490" s="1" t="s">
-        <v>3273</v>
+        <v>3272</v>
       </c>
       <c r="D490" s="1" t="s">
         <v>115</v>
@@ -81239,7 +81263,7 @@
         <v>694</v>
       </c>
       <c r="E491" s="1" t="s">
-        <v>3235</v>
+        <v>3234</v>
       </c>
       <c r="F491" s="1" t="s">
         <v>35</v>
@@ -81260,13 +81284,13 @@
         <v>2814</v>
       </c>
       <c r="B492" s="1" t="s">
-        <v>3334</v>
+        <v>3333</v>
       </c>
       <c r="C492" s="1" t="s">
         <v>1236</v>
       </c>
       <c r="D492" s="1" t="s">
-        <v>3271</v>
+        <v>3270</v>
       </c>
       <c r="E492" s="1" t="s">
         <v>97</v>
@@ -81305,7 +81329,7 @@
         <v>36</v>
       </c>
       <c r="G493" s="1" t="s">
-        <v>3488</v>
+        <v>3487</v>
       </c>
       <c r="H493" s="1" t="s">
         <v>1659</v>
@@ -81337,7 +81361,7 @@
         <v>35</v>
       </c>
       <c r="G494" s="1" t="s">
-        <v>3481</v>
+        <v>3480</v>
       </c>
       <c r="H494" s="1" t="s">
         <v>1659</v>
@@ -81369,7 +81393,7 @@
         <v>36</v>
       </c>
       <c r="G495" s="1" t="s">
-        <v>3482</v>
+        <v>3481</v>
       </c>
       <c r="H495" s="1" t="s">
         <v>1659</v>
@@ -81401,7 +81425,7 @@
         <v>36</v>
       </c>
       <c r="G496" s="1" t="s">
-        <v>3486</v>
+        <v>3485</v>
       </c>
       <c r="H496" s="1" t="s">
         <v>1659</v>
@@ -81463,7 +81487,7 @@
         <v>35</v>
       </c>
       <c r="G498" s="1" t="s">
-        <v>3483</v>
+        <v>3482</v>
       </c>
       <c r="H498" s="1" t="s">
         <v>1659</v>
@@ -81480,7 +81504,7 @@
         <v>2807</v>
       </c>
       <c r="B499" s="1" t="s">
-        <v>3333</v>
+        <v>3332</v>
       </c>
       <c r="C499" s="1" t="s">
         <v>832</v>
@@ -81543,7 +81567,7 @@
         <v>1741</v>
       </c>
       <c r="C501" s="1" t="s">
-        <v>3410</v>
+        <v>3409</v>
       </c>
       <c r="D501" s="1" t="s">
         <v>679</v>
@@ -82125,7 +82149,7 @@
         <v>35</v>
       </c>
       <c r="G520" s="1" t="s">
-        <v>3456</v>
+        <v>3455</v>
       </c>
       <c r="H520" s="1" t="s">
         <v>1659</v>
@@ -82157,7 +82181,7 @@
         <v>36</v>
       </c>
       <c r="G521" s="1" t="s">
-        <v>3491</v>
+        <v>3490</v>
       </c>
       <c r="H521" s="1" t="s">
         <v>1659</v>
@@ -82279,7 +82303,7 @@
         <v>36</v>
       </c>
       <c r="G525" s="1" t="s">
-        <v>3484</v>
+        <v>3483</v>
       </c>
       <c r="H525" s="1" t="s">
         <v>1659</v>
@@ -82311,7 +82335,7 @@
         <v>36</v>
       </c>
       <c r="G526" s="1" t="s">
-        <v>3490</v>
+        <v>3489</v>
       </c>
       <c r="H526" s="1" t="s">
         <v>1659</v>
@@ -82320,22 +82344,22 @@
         <v>594</v>
       </c>
       <c r="J526" s="1" t="s">
-        <v>3428</v>
+        <v>3427</v>
       </c>
     </row>
     <row r="527" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A527" s="1"/>
       <c r="B527" s="1" t="s">
+        <v>3428</v>
+      </c>
+      <c r="C527" s="1" t="s">
         <v>3429</v>
       </c>
-      <c r="C527" s="1" t="s">
+      <c r="D527" s="1" t="s">
         <v>3430</v>
       </c>
-      <c r="D527" s="1" t="s">
+      <c r="E527" s="1" t="s">
         <v>3431</v>
-      </c>
-      <c r="E527" s="1" t="s">
-        <v>3432</v>
       </c>
       <c r="F527" s="1"/>
       <c r="G527" s="1"/>
@@ -82350,16 +82374,16 @@
     <row r="528" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A528" s="1"/>
       <c r="B528" s="1" t="s">
+        <v>3432</v>
+      </c>
+      <c r="C528" s="1" t="s">
         <v>3433</v>
       </c>
-      <c r="C528" s="1" t="s">
+      <c r="D528" s="1" t="s">
         <v>3434</v>
       </c>
-      <c r="D528" s="1" t="s">
+      <c r="E528" s="1" t="s">
         <v>3435</v>
-      </c>
-      <c r="E528" s="1" t="s">
-        <v>3436</v>
       </c>
       <c r="F528" s="1"/>
       <c r="G528" s="1"/>
@@ -82374,7 +82398,7 @@
     <row r="529" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A529" s="1"/>
       <c r="B529" s="1" t="s">
-        <v>3437</v>
+        <v>3436</v>
       </c>
       <c r="C529" s="1">
         <v>0.5</v>
@@ -82398,16 +82422,16 @@
     <row r="530" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A530" s="1"/>
       <c r="B530" s="1" t="s">
+        <v>3437</v>
+      </c>
+      <c r="C530" s="1" t="s">
         <v>3438</v>
       </c>
-      <c r="C530" s="1" t="s">
+      <c r="D530" s="1" t="s">
         <v>3439</v>
       </c>
-      <c r="D530" s="1" t="s">
+      <c r="E530" s="1" t="s">
         <v>3440</v>
-      </c>
-      <c r="E530" s="1" t="s">
-        <v>3441</v>
       </c>
       <c r="F530" s="1"/>
       <c r="G530" s="1"/>

</xml_diff>